<commit_message>
changed 47, 52, and lots of things
</commit_message>
<xml_diff>
--- a/db/data/projects.xlsx
+++ b/db/data/projects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pradeep\Desktop\storemgmt\db\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931EA459-55AC-4A76-9CC1-F1B29583553D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082C21F6-3A1E-4C9D-98B8-43C7209862D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2355" yWindow="690" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11295" yWindow="1905" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="1" r:id="rId1"/>
@@ -307,9 +307,6 @@
     <t>ध्यानुङ्ग लिफ्ट खानेपानी आयोजना</t>
   </si>
   <si>
-    <t>Ghyanung Lift Water Supply and Sanitation Project</t>
-  </si>
-  <si>
     <t>खाल्टे  खानेपानी आयोजना</t>
   </si>
   <si>
@@ -605,6 +602,9 @@
   </si>
   <si>
     <t>project_status</t>
+  </si>
+  <si>
+    <t>Dhenung Lift Water Supply and Sanitation Project</t>
   </si>
 </sst>
 </file>
@@ -986,7 +986,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -1627,7 +1627,7 @@
         <v>94</v>
       </c>
       <c r="D47" t="s">
-        <v>95</v>
+        <v>194</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -1638,10 +1638,10 @@
         <v>47</v>
       </c>
       <c r="C48" t="s">
+        <v>95</v>
+      </c>
+      <c r="D48" t="s">
         <v>96</v>
-      </c>
-      <c r="D48" t="s">
-        <v>97</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -1652,10 +1652,10 @@
         <v>48</v>
       </c>
       <c r="C49" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" t="s">
         <v>98</v>
-      </c>
-      <c r="D49" t="s">
-        <v>99</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -1666,10 +1666,10 @@
         <v>49</v>
       </c>
       <c r="C50" t="s">
+        <v>99</v>
+      </c>
+      <c r="D50" t="s">
         <v>100</v>
-      </c>
-      <c r="D50" t="s">
-        <v>101</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -1680,10 +1680,10 @@
         <v>50</v>
       </c>
       <c r="C51" t="s">
+        <v>101</v>
+      </c>
+      <c r="D51" t="s">
         <v>102</v>
-      </c>
-      <c r="D51" t="s">
-        <v>103</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -1694,10 +1694,10 @@
         <v>51</v>
       </c>
       <c r="C52" t="s">
+        <v>103</v>
+      </c>
+      <c r="D52" t="s">
         <v>104</v>
-      </c>
-      <c r="D52" t="s">
-        <v>105</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -1708,10 +1708,10 @@
         <v>52</v>
       </c>
       <c r="C53" t="s">
+        <v>105</v>
+      </c>
+      <c r="D53" t="s">
         <v>106</v>
-      </c>
-      <c r="D53" t="s">
-        <v>107</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -1722,10 +1722,10 @@
         <v>53</v>
       </c>
       <c r="C54" t="s">
+        <v>107</v>
+      </c>
+      <c r="D54" t="s">
         <v>108</v>
-      </c>
-      <c r="D54" t="s">
-        <v>109</v>
       </c>
       <c r="E54">
         <v>0</v>
@@ -1736,10 +1736,10 @@
         <v>54</v>
       </c>
       <c r="C55" t="s">
+        <v>109</v>
+      </c>
+      <c r="D55" t="s">
         <v>110</v>
-      </c>
-      <c r="D55" t="s">
-        <v>111</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -1750,10 +1750,10 @@
         <v>55</v>
       </c>
       <c r="C56" t="s">
+        <v>111</v>
+      </c>
+      <c r="D56" t="s">
         <v>112</v>
-      </c>
-      <c r="D56" t="s">
-        <v>113</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -1764,10 +1764,10 @@
         <v>56</v>
       </c>
       <c r="C57" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" t="s">
         <v>114</v>
-      </c>
-      <c r="D57" t="s">
-        <v>115</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -1778,10 +1778,10 @@
         <v>57</v>
       </c>
       <c r="C58" t="s">
+        <v>115</v>
+      </c>
+      <c r="D58" t="s">
         <v>116</v>
-      </c>
-      <c r="D58" t="s">
-        <v>117</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -1792,10 +1792,10 @@
         <v>58</v>
       </c>
       <c r="C59" t="s">
+        <v>117</v>
+      </c>
+      <c r="D59" t="s">
         <v>118</v>
-      </c>
-      <c r="D59" t="s">
-        <v>119</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -1806,10 +1806,10 @@
         <v>59</v>
       </c>
       <c r="C60" t="s">
+        <v>119</v>
+      </c>
+      <c r="D60" t="s">
         <v>120</v>
-      </c>
-      <c r="D60" t="s">
-        <v>121</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -1820,10 +1820,10 @@
         <v>60</v>
       </c>
       <c r="C61" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" t="s">
         <v>122</v>
-      </c>
-      <c r="D61" t="s">
-        <v>123</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -1834,10 +1834,10 @@
         <v>61</v>
       </c>
       <c r="C62" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" t="s">
         <v>124</v>
-      </c>
-      <c r="D62" t="s">
-        <v>125</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -1848,10 +1848,10 @@
         <v>62</v>
       </c>
       <c r="C63" t="s">
+        <v>125</v>
+      </c>
+      <c r="D63" t="s">
         <v>126</v>
-      </c>
-      <c r="D63" t="s">
-        <v>127</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -1862,10 +1862,10 @@
         <v>63</v>
       </c>
       <c r="C64" t="s">
+        <v>127</v>
+      </c>
+      <c r="D64" t="s">
         <v>128</v>
-      </c>
-      <c r="D64" t="s">
-        <v>129</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -1876,10 +1876,10 @@
         <v>64</v>
       </c>
       <c r="C65" t="s">
+        <v>129</v>
+      </c>
+      <c r="D65" t="s">
         <v>130</v>
-      </c>
-      <c r="D65" t="s">
-        <v>131</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -1890,10 +1890,10 @@
         <v>65</v>
       </c>
       <c r="C66" t="s">
+        <v>131</v>
+      </c>
+      <c r="D66" t="s">
         <v>132</v>
-      </c>
-      <c r="D66" t="s">
-        <v>133</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -1904,10 +1904,10 @@
         <v>66</v>
       </c>
       <c r="C67" t="s">
+        <v>133</v>
+      </c>
+      <c r="D67" t="s">
         <v>134</v>
-      </c>
-      <c r="D67" t="s">
-        <v>135</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -1918,10 +1918,10 @@
         <v>67</v>
       </c>
       <c r="C68" t="s">
+        <v>135</v>
+      </c>
+      <c r="D68" t="s">
         <v>136</v>
-      </c>
-      <c r="D68" t="s">
-        <v>137</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -1932,10 +1932,10 @@
         <v>68</v>
       </c>
       <c r="C69" t="s">
+        <v>137</v>
+      </c>
+      <c r="D69" t="s">
         <v>138</v>
-      </c>
-      <c r="D69" t="s">
-        <v>139</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -1946,10 +1946,10 @@
         <v>69</v>
       </c>
       <c r="C70" t="s">
+        <v>139</v>
+      </c>
+      <c r="D70" t="s">
         <v>140</v>
-      </c>
-      <c r="D70" t="s">
-        <v>141</v>
       </c>
       <c r="E70">
         <v>0</v>
@@ -1960,10 +1960,10 @@
         <v>70</v>
       </c>
       <c r="C71" t="s">
+        <v>141</v>
+      </c>
+      <c r="D71" t="s">
         <v>142</v>
-      </c>
-      <c r="D71" t="s">
-        <v>143</v>
       </c>
       <c r="E71">
         <v>0</v>
@@ -1974,10 +1974,10 @@
         <v>71</v>
       </c>
       <c r="C72" t="s">
+        <v>143</v>
+      </c>
+      <c r="D72" t="s">
         <v>144</v>
-      </c>
-      <c r="D72" t="s">
-        <v>145</v>
       </c>
       <c r="E72">
         <v>0</v>
@@ -1988,10 +1988,10 @@
         <v>72</v>
       </c>
       <c r="C73" t="s">
+        <v>145</v>
+      </c>
+      <c r="D73" t="s">
         <v>146</v>
-      </c>
-      <c r="D73" t="s">
-        <v>147</v>
       </c>
       <c r="E73">
         <v>0</v>
@@ -2002,10 +2002,10 @@
         <v>73</v>
       </c>
       <c r="C74" t="s">
+        <v>147</v>
+      </c>
+      <c r="D74" t="s">
         <v>148</v>
-      </c>
-      <c r="D74" t="s">
-        <v>149</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -2016,10 +2016,10 @@
         <v>74</v>
       </c>
       <c r="C75" t="s">
+        <v>149</v>
+      </c>
+      <c r="D75" t="s">
         <v>150</v>
-      </c>
-      <c r="D75" t="s">
-        <v>151</v>
       </c>
       <c r="E75">
         <v>0</v>
@@ -2030,10 +2030,10 @@
         <v>75</v>
       </c>
       <c r="C76" t="s">
+        <v>151</v>
+      </c>
+      <c r="D76" t="s">
         <v>152</v>
-      </c>
-      <c r="D76" t="s">
-        <v>153</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -2044,10 +2044,10 @@
         <v>76</v>
       </c>
       <c r="C77" t="s">
+        <v>153</v>
+      </c>
+      <c r="D77" t="s">
         <v>154</v>
-      </c>
-      <c r="D77" t="s">
-        <v>155</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -2058,10 +2058,10 @@
         <v>77</v>
       </c>
       <c r="C78" t="s">
+        <v>155</v>
+      </c>
+      <c r="D78" t="s">
         <v>156</v>
-      </c>
-      <c r="D78" t="s">
-        <v>157</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -2072,10 +2072,10 @@
         <v>78</v>
       </c>
       <c r="C79" t="s">
+        <v>157</v>
+      </c>
+      <c r="D79" t="s">
         <v>158</v>
-      </c>
-      <c r="D79" t="s">
-        <v>159</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -2086,10 +2086,10 @@
         <v>79</v>
       </c>
       <c r="C80" t="s">
+        <v>159</v>
+      </c>
+      <c r="D80" t="s">
         <v>160</v>
-      </c>
-      <c r="D80" t="s">
-        <v>161</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -2100,10 +2100,10 @@
         <v>80</v>
       </c>
       <c r="C81" t="s">
+        <v>161</v>
+      </c>
+      <c r="D81" t="s">
         <v>162</v>
-      </c>
-      <c r="D81" t="s">
-        <v>163</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -2114,10 +2114,10 @@
         <v>81</v>
       </c>
       <c r="C82" t="s">
+        <v>163</v>
+      </c>
+      <c r="D82" t="s">
         <v>164</v>
-      </c>
-      <c r="D82" t="s">
-        <v>165</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -2128,10 +2128,10 @@
         <v>82</v>
       </c>
       <c r="C83" t="s">
+        <v>165</v>
+      </c>
+      <c r="D83" t="s">
         <v>166</v>
-      </c>
-      <c r="D83" t="s">
-        <v>167</v>
       </c>
       <c r="E83">
         <v>0</v>
@@ -2142,10 +2142,10 @@
         <v>83</v>
       </c>
       <c r="C84" t="s">
+        <v>167</v>
+      </c>
+      <c r="D84" t="s">
         <v>168</v>
-      </c>
-      <c r="D84" t="s">
-        <v>169</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -2156,10 +2156,10 @@
         <v>84</v>
       </c>
       <c r="C85" t="s">
+        <v>169</v>
+      </c>
+      <c r="D85" t="s">
         <v>170</v>
-      </c>
-      <c r="D85" t="s">
-        <v>171</v>
       </c>
       <c r="E85">
         <v>0</v>
@@ -2170,10 +2170,10 @@
         <v>85</v>
       </c>
       <c r="C86" t="s">
+        <v>171</v>
+      </c>
+      <c r="D86" t="s">
         <v>172</v>
-      </c>
-      <c r="D86" t="s">
-        <v>173</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -2184,10 +2184,10 @@
         <v>86</v>
       </c>
       <c r="C87" t="s">
+        <v>173</v>
+      </c>
+      <c r="D87" t="s">
         <v>174</v>
-      </c>
-      <c r="D87" t="s">
-        <v>175</v>
       </c>
       <c r="E87">
         <v>0</v>
@@ -2198,10 +2198,10 @@
         <v>87</v>
       </c>
       <c r="C88" t="s">
+        <v>175</v>
+      </c>
+      <c r="D88" t="s">
         <v>176</v>
-      </c>
-      <c r="D88" t="s">
-        <v>177</v>
       </c>
       <c r="E88">
         <v>0</v>
@@ -2212,10 +2212,10 @@
         <v>88</v>
       </c>
       <c r="C89" t="s">
+        <v>177</v>
+      </c>
+      <c r="D89" t="s">
         <v>178</v>
-      </c>
-      <c r="D89" t="s">
-        <v>179</v>
       </c>
       <c r="E89">
         <v>0</v>
@@ -2226,10 +2226,10 @@
         <v>89</v>
       </c>
       <c r="C90" t="s">
+        <v>179</v>
+      </c>
+      <c r="D90" t="s">
         <v>180</v>
-      </c>
-      <c r="D90" t="s">
-        <v>181</v>
       </c>
       <c r="E90">
         <v>0</v>
@@ -2240,10 +2240,10 @@
         <v>90</v>
       </c>
       <c r="C91" t="s">
+        <v>181</v>
+      </c>
+      <c r="D91" t="s">
         <v>182</v>
-      </c>
-      <c r="D91" t="s">
-        <v>183</v>
       </c>
       <c r="E91">
         <v>0</v>
@@ -2254,10 +2254,10 @@
         <v>91</v>
       </c>
       <c r="C92" t="s">
+        <v>183</v>
+      </c>
+      <c r="D92" t="s">
         <v>184</v>
-      </c>
-      <c r="D92" t="s">
-        <v>185</v>
       </c>
       <c r="E92">
         <v>0</v>
@@ -2268,10 +2268,10 @@
         <v>92</v>
       </c>
       <c r="C93" t="s">
+        <v>185</v>
+      </c>
+      <c r="D93" t="s">
         <v>186</v>
-      </c>
-      <c r="D93" t="s">
-        <v>187</v>
       </c>
       <c r="E93">
         <v>0</v>
@@ -2282,10 +2282,10 @@
         <v>93</v>
       </c>
       <c r="C94" t="s">
+        <v>187</v>
+      </c>
+      <c r="D94" t="s">
         <v>188</v>
-      </c>
-      <c r="D94" t="s">
-        <v>189</v>
       </c>
       <c r="E94">
         <v>0</v>
@@ -2296,10 +2296,10 @@
         <v>94</v>
       </c>
       <c r="C95" t="s">
+        <v>189</v>
+      </c>
+      <c r="D95" t="s">
         <v>190</v>
-      </c>
-      <c r="D95" t="s">
-        <v>191</v>
       </c>
       <c r="E95">
         <v>0</v>
@@ -2310,10 +2310,10 @@
         <v>95</v>
       </c>
       <c r="C96" t="s">
+        <v>191</v>
+      </c>
+      <c r="D96" t="s">
         <v>192</v>
-      </c>
-      <c r="D96" t="s">
-        <v>193</v>
       </c>
       <c r="E96">
         <v>0</v>

</xml_diff>